<commit_message>
[UPD] 16.0 sync from gitlab
</commit_message>
<xml_diff>
--- a/import_template_partner/data/template_partner.xlsx
+++ b/import_template_partner/data/template_partner.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="property_product_pricelist" vbProcedure="false">Hoja1!$AH$2</definedName>
+    <definedName function="false" hidden="false" name="property_product_pricelist" vbProcedure="false">Hoja1!$AE$2</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="80">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -85,19 +85,13 @@
     <t xml:space="preserve">comment</t>
   </si>
   <si>
-    <t xml:space="preserve">customer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">supplier</t>
-  </si>
-  <si>
     <t xml:space="preserve">agent</t>
   </si>
   <si>
     <t xml:space="preserve">agent_type</t>
   </si>
   <si>
-    <t xml:space="preserve">commission</t>
+    <t xml:space="preserve">commission_id</t>
   </si>
   <si>
     <t xml:space="preserve">settlement</t>
@@ -106,7 +100,7 @@
     <t xml:space="preserve">user_id</t>
   </si>
   <si>
-    <t xml:space="preserve">invoice_group_method_id</t>
+    <t xml:space="preserve">sale_invoicing_grouping_criteria_id</t>
   </si>
   <si>
     <t xml:space="preserve">property_payment_term_id</t>
@@ -121,15 +115,9 @@
     <t xml:space="preserve">supplier_payment_mode_id</t>
   </si>
   <si>
-    <t xml:space="preserve">default_supplierinfo_multiple_discount</t>
-  </si>
-  <si>
     <t xml:space="preserve">property_product_pricelist</t>
   </si>
   <si>
-    <t xml:space="preserve">supplier_pricelist_id</t>
-  </si>
-  <si>
     <t xml:space="preserve">ref</t>
   </si>
   <si>
@@ -193,9 +181,6 @@
     <t xml:space="preserve">Notes from tests.</t>
   </si>
   <si>
-    <t xml:space="preserve">True</t>
-  </si>
-  <si>
     <t xml:space="preserve">María Luisa Martín</t>
   </si>
   <si>
@@ -208,13 +193,7 @@
     <t xml:space="preserve">30 Días</t>
   </si>
   <si>
-    <t xml:space="preserve">5+3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tarifa pública</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarifa prueba 1</t>
   </si>
   <si>
     <t xml:space="preserve">Ref 1</t>
@@ -294,7 +273,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;"/>
-    <numFmt numFmtId="167" formatCode="DD/MM/YY"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yy"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -393,23 +372,23 @@
     </xf>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="false"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3" customBuiltin="false"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6" customBuiltin="false"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4" customBuiltin="false"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7" customBuiltin="false"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5" customBuiltin="false"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AQ6"/>
-  <sheetFormatPr defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AM6"/>
+  <sheetFormatPr defaultColWidth="8.91015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.28"/>
@@ -419,32 +398,26 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="24.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8.1"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="12" min="9" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="15.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="8.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="9" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="15.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="11.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="40.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="20" style="0" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="19.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="26" style="0" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="28.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="20.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="37.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="25.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="35.42"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="35" min="34" style="0" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="25.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="21.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="14.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="29.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1023" min="41" style="0" width="8.89"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="1024" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="19.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="28.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="20.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="37.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="25.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="25.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="0" width="21.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="14.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="29.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1020" min="1020" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1021" style="0" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -526,7 +499,7 @@
       <c r="AA1" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="0" t="s">
+      <c r="AB1" s="3" t="s">
         <v>27</v>
       </c>
       <c r="AC1" s="0" t="s">
@@ -535,16 +508,16 @@
       <c r="AD1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="0" t="s">
+      <c r="AE1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AF1" s="0" t="s">
         <v>31</v>
       </c>
       <c r="AG1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AH1" s="0" t="s">
         <v>33</v>
       </c>
       <c r="AI1" s="3" t="s">
@@ -556,56 +529,44 @@
       <c r="AK1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="0" t="s">
+      <c r="AL1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AM1" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="0" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="5"/>
       <c r="L2" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="0" t="n">
@@ -615,80 +576,71 @@
         <v>666555666</v>
       </c>
       <c r="Q2" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="R2" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="S2" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="T2" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y2" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="R2" s="0" t="s">
+      <c r="Z2" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="S2" s="0" t="s">
+      <c r="AA2" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="T2" s="0" t="s">
+      <c r="AB2" s="0" t="s">
         <v>55</v>
       </c>
-      <c r="U2" s="0" t="s">
+      <c r="AE2" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="AA2" s="3" t="s">
+      <c r="AF2" s="0" t="s">
         <v>57</v>
       </c>
-      <c r="AB2" s="0" t="s">
+      <c r="AG2" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="AC2" s="0" t="s">
+      <c r="AH2" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="AD2" s="0" t="s">
+      <c r="AI2" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="AG2" s="0" t="s">
+      <c r="AJ2" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="AH2" s="0" t="s">
+      <c r="AK2" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="AI2" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="AJ2" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="AK2" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="AL2" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="AM2" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN2" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="AO2" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="AP2" s="6" t="n">
+      <c r="AL2" s="6" t="n">
         <v>44197</v>
       </c>
-      <c r="AQ2" s="0" t="n">
+      <c r="AM2" s="0" t="n">
         <v>8888</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -701,76 +653,73 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="K4" s="1"/>
       <c r="M4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="4" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="H5" s="4"/>
       <c r="K5" s="5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="U5" s="0" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="4" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>11111</v>
@@ -778,22 +727,19 @@
       <c r="K6" s="5"/>
       <c r="L6" s="1"/>
       <c r="M6" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="U6" s="0" t="s">
-        <v>56</v>
+        <v>77</v>
+      </c>
+      <c r="V6" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="W6" s="0" t="s">
+        <v>78</v>
       </c>
       <c r="X6" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y6" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="Z6" s="0" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>